<commit_message>
Commit before local delete
</commit_message>
<xml_diff>
--- a/data/CABG Hyperglycemia Variable List.xlsx
+++ b/data/CABG Hyperglycemia Variable List.xlsx
@@ -3,10 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1385B5C-0657-407E-BC90-214C39F573E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69B95A4-A98E-4376-8693-3EE9F6BF9223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="17" activeTab="20" xr2:uid="{D170740D-F730-4FE0-A2DA-00C8EA3E9EA2}"/>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="23" activeTab="25" xr2:uid="{18D90FB9-8B94-4B85-AE0C-47B2E521BCF3}"/>
+    <workbookView xWindow="19090" yWindow="-6530" windowWidth="19420" windowHeight="10420" firstSheet="26" activeTab="27" xr2:uid="{18D90FB9-8B94-4B85-AE0C-47B2E521BCF3}"/>
   </bookViews>
   <sheets>
     <sheet name="or_to_icu" sheetId="1" state="hidden" r:id="rId1"/>
@@ -35,8 +34,10 @@
     <sheet name="hilic_feature_2" sheetId="25" r:id="rId24"/>
     <sheet name="C18_Mummichog Metabolite Match" sheetId="26" r:id="rId25"/>
     <sheet name="HIL_Mummichog Metabolite Match" sheetId="27" r:id="rId26"/>
-    <sheet name="aha glucose" sheetId="5" state="hidden" r:id="rId27"/>
-    <sheet name="aha patient" sheetId="6" state="hidden" r:id="rId28"/>
+    <sheet name="Sig_Annotation_negative_AllVisi" sheetId="31" r:id="rId27"/>
+    <sheet name="Sig_Annotation_positive_AllVisi" sheetId="32" r:id="rId28"/>
+    <sheet name="aha glucose" sheetId="5" state="hidden" r:id="rId29"/>
+    <sheet name="aha patient" sheetId="6" state="hidden" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'METACABG 20230706'!$B$1:$J$505</definedName>
@@ -97,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7147" uniqueCount="4201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7205" uniqueCount="4225">
   <si>
     <t>variable</t>
   </si>
@@ -12762,6 +12763,84 @@
   </si>
   <si>
     <t>Number of POCT blood glucose measurements &gt;= 189 mg/dL</t>
+  </si>
+  <si>
+    <t>~/data/chd07_metabolites annotated using multiple databases.R</t>
+  </si>
+  <si>
+    <t>Sig_Annotation_negative_AllVisits</t>
+  </si>
+  <si>
+    <t>Sig_Annotation_positive_AllVisits</t>
+  </si>
+  <si>
+    <t>From New 2023 Analysis\Full Annotator</t>
+  </si>
+  <si>
+    <t>chemical_ID</t>
+  </si>
+  <si>
+    <t>annotation_confidence_score</t>
+  </si>
+  <si>
+    <t>theoretical_mz</t>
+  </si>
+  <si>
+    <t>delta_ppm</t>
+  </si>
+  <si>
+    <t>formula</t>
+  </si>
+  <si>
+    <t>mono_isotopic_mass</t>
+  </si>
+  <si>
+    <t>adduct</t>
+  </si>
+  <si>
+    <t>p_value</t>
+  </si>
+  <si>
+    <t>adjusted_p_value</t>
+  </si>
+  <si>
+    <t>max_fold_change_log2</t>
+  </si>
+  <si>
+    <t>This is the database ID for the metabolite: Those that begin with C are KEGG, HMDB (Human Metabolome), LM (LipidMaps), and T3D (Toxin)</t>
+  </si>
+  <si>
+    <t>the perfect mz if you were to add elements weight together</t>
+  </si>
+  <si>
+    <t>m/z drift from the detected m/z to the theoretical m/z in parts per million</t>
+  </si>
+  <si>
+    <t>metabolite name</t>
+  </si>
+  <si>
+    <t>chemical formula of the metabolite</t>
+  </si>
+  <si>
+    <t>mass of the ion containing principal ions only</t>
+  </si>
+  <si>
+    <t>unadjusted p-value</t>
+  </si>
+  <si>
+    <t>If this is from mummichog, this is the computed p value after 1000 permutations</t>
+  </si>
+  <si>
+    <t>score-based annotation using multiple criteria (m/z, time, isotope, adduct, intensity, network, pathway). 3 is the highest, 0 is the lowest, see criteria below
+Confidence level assignment: Each chemical is categorized as no confidence (0), low confidence (1), medium confidence, (2) and high confidence (3) based on the following criteria:
+Score is greater than zero
+Presence of required adducts/forms specified by the user for assignment to high confidence categories (e.g. M+H)
+N, O, P, S/C ratio checks
+Hydrogen/Carbon ratio check
+Abundance ratio checks for isotopes, multimers (dimers and trimers), and multiply charged adducts with respect to the singly charged adducts and ions according to heuristic rules.</t>
+  </si>
+  <si>
+    <t>Log2 fold change of the metabolite in the comparison in question ( e.g. Case v Control, Visit 1 vs Visit 2 etc)</t>
   </si>
 </sst>
 </file>
@@ -12876,7 +12955,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -12890,6 +12969,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -16114,6 +16194,245 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F05B6D-AC46-417B-8FF1-D00A90A9920A}">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.90625" customWidth="1"/>
+    <col min="2" max="2" width="23.7265625" customWidth="1"/>
+    <col min="10" max="10" width="10.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4205</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4206</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>4223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4150</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4207</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4216</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4208</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4217</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4164</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4218</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4209</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4219</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4210</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4220</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4211</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4212</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4221</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4213</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4222</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4214</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4224</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C031532-DB6E-4BCE-AA3A-172D0AF83212}">
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.90625" customWidth="1"/>
+    <col min="2" max="2" width="23.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4205</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4206</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>4223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4150</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4208</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4217</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4164</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4218</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4209</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4219</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4210</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4220</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4211</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4212</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4221</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4213</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4222</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4214</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4224</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F730E738-71E8-4BB9-9BDD-FAFBA3CE3EC3}">
   <dimension ref="A1:B146"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -17174,269 +17493,6 @@
     <row r="146" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>717</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A7ED6AA-780D-40B6-8131-5D17C4E940B1}">
-  <dimension ref="A1:B32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="90.08984375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>622</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>623</v>
-      </c>
-      <c r="B4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>546</v>
-      </c>
-      <c r="B5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>624</v>
-      </c>
-      <c r="B6" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>625</v>
-      </c>
-      <c r="B7" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>513</v>
-      </c>
-      <c r="B8" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>511</v>
-      </c>
-      <c r="B9" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>626</v>
-      </c>
-      <c r="B10" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>627</v>
-      </c>
-      <c r="B11" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>628</v>
-      </c>
-      <c r="B12" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>629</v>
-      </c>
-      <c r="B13" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>630</v>
-      </c>
-      <c r="B14" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>631</v>
-      </c>
-      <c r="B15" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>632</v>
-      </c>
-      <c r="B16" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>633</v>
-      </c>
-      <c r="B17" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>634</v>
-      </c>
-      <c r="B18" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>635</v>
-      </c>
-      <c r="B19" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>636</v>
-      </c>
-      <c r="B20" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>637</v>
-      </c>
-      <c r="B21" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>638</v>
-      </c>
-      <c r="B22" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>639</v>
-      </c>
-      <c r="B23" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>641</v>
-      </c>
-      <c r="B25" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>642</v>
-      </c>
-      <c r="B26" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>643</v>
-      </c>
-      <c r="B27" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>644</v>
-      </c>
-      <c r="B28" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>645</v>
-      </c>
-      <c r="B29" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>646</v>
-      </c>
-      <c r="B30" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>647</v>
-      </c>
-      <c r="B31" t="s">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>648</v>
-      </c>
-      <c r="B32" t="s">
-        <v>665</v>
       </c>
     </row>
   </sheetData>
@@ -18952,9 +19008,272 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A7ED6AA-780D-40B6-8131-5D17C4E940B1}">
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="90.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>623</v>
+      </c>
+      <c r="B4" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>546</v>
+      </c>
+      <c r="B5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>624</v>
+      </c>
+      <c r="B6" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>625</v>
+      </c>
+      <c r="B7" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>513</v>
+      </c>
+      <c r="B8" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>511</v>
+      </c>
+      <c r="B9" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>626</v>
+      </c>
+      <c r="B10" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>627</v>
+      </c>
+      <c r="B11" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>628</v>
+      </c>
+      <c r="B12" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>629</v>
+      </c>
+      <c r="B13" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>630</v>
+      </c>
+      <c r="B14" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>631</v>
+      </c>
+      <c r="B15" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>632</v>
+      </c>
+      <c r="B16" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>633</v>
+      </c>
+      <c r="B17" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>634</v>
+      </c>
+      <c r="B18" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>635</v>
+      </c>
+      <c r="B19" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>636</v>
+      </c>
+      <c r="B20" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>637</v>
+      </c>
+      <c r="B21" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>638</v>
+      </c>
+      <c r="B22" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>639</v>
+      </c>
+      <c r="B23" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>641</v>
+      </c>
+      <c r="B25" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>642</v>
+      </c>
+      <c r="B26" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>643</v>
+      </c>
+      <c r="B27" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>644</v>
+      </c>
+      <c r="B28" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>645</v>
+      </c>
+      <c r="B29" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>646</v>
+      </c>
+      <c r="B30" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>647</v>
+      </c>
+      <c r="B31" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>648</v>
+      </c>
+      <c r="B32" t="s">
+        <v>665</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08C9B308-162A-4FA9-98F4-5823503BDBEE}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -19137,6 +19456,28 @@
       </c>
       <c r="C21" t="s">
         <v>4196</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>4202</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4204</v>
+      </c>
+      <c r="C22" t="s">
+        <v>4201</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>4203</v>
+      </c>
+      <c r="B23" t="s">
+        <v>4204</v>
+      </c>
+      <c r="C23" t="s">
+        <v>4201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>